<commit_message>
Refine payroll input menu and bonus settings
</commit_message>
<xml_diff>
--- a/docs/manual_payroll_ses_ja_zh.xlsx
+++ b/docs/manual_payroll_ses_ja_zh.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目次" sheetId="1" r:id="R92828e594d38493e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_JA" sheetId="2" r:id="Rf43a78f5ba2e4061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_ZH" sheetId="3" r:id="R5e43377588944627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_JA" sheetId="4" r:id="R461dc2b49fc443ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_ZH" sheetId="5" r:id="R7e1f0750cd324030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目次" sheetId="1" r:id="R53edcda026ec49bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_JA" sheetId="2" r:id="R31b16f3e071a4a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_ZH" sheetId="3" r:id="R596937e65c6f4d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_JA" sheetId="4" r:id="R1798e802ae414602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_ZH" sheetId="5" r:id="R0c6ed986ab2e4167"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -532,7 +532,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>「給与管理」から社員一覧を開きます。</x:v>
+        <x:v>「給与管理」から「社員管理」を開きます。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -570,31 +570,31 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="17" t="str">
-        <x:v>3. 年度・料率管理</x:v>
-      </x:c>
-      <x:c r="B14" s="18" t="str"/>
-      <x:c r="C14" s="15" t="str"/>
+        <x:v>2. 社員管理</x:v>
+      </x:c>
+      <x:c r="B14" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="str">
+        <x:v>賞与あり/なしを社員ごとに設定できます。賞与ありの場合、最大3回まで支給月と金額を登録できます。</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>3. 年度・料率管理</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C15" s="15" t="str">
-        <x:v>税金、社会保険料率は年度ごとに登録します。</x:v>
-      </x:c>
+      <x:c r="B15" s="18" t="str"/>
+      <x:c r="C15" s="15" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
         <x:v>3. 年度・料率管理</x:v>
       </x:c>
       <x:c r="B16" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C16" s="15" t="str">
-        <x:v>健康・介護保険料率、厚生年金保険料率、雇用保険料率、子ども・子育て支援金を分けて入力します。</x:v>
+        <x:v>税金、社会保険料率は年度ごとに登録します。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -602,10 +602,10 @@
         <x:v>3. 年度・料率管理</x:v>
       </x:c>
       <x:c r="B17" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C17" s="15" t="str">
-        <x:v>小数点は6桁まで入力できます。</x:v>
+        <x:v>健康・介護保険料率、厚生年金保険料率、雇用保険料率、子ども・子育て支援金を分けて入力します。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -613,39 +613,39 @@
         <x:v>3. 年度・料率管理</x:v>
       </x:c>
       <x:c r="B18" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C18" s="15" t="str">
-        <x:v>住民税は給与入力時に社員ごと、月ごとに入力します。</x:v>
+        <x:v>小数点は6桁まで入力できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>4. 所得税表</x:v>
-      </x:c>
-      <x:c r="B19" s="18" t="str"/>
-      <x:c r="C19" s="15" t="str"/>
+        <x:v>3. 年度・料率管理</x:v>
+      </x:c>
+      <x:c r="B19" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>住民税は給与入力時に社員ごと、月ごとに入力します。</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C20" s="15" t="str">
-        <x:v>所得税表CSVをインポートします。</x:v>
-      </x:c>
+      <x:c r="B20" s="18" t="str"/>
+      <x:c r="C20" s="15" t="str"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
-        <x:v>CSV形式は `fiscalYear,dependentCount,minTaxable,maxTaxable,taxAmount` です。</x:v>
+        <x:v>所得税表CSVをインポートします。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -653,39 +653,39 @@
         <x:v>4. 所得税表</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="15" t="str">
-        <x:v>給与計算時は年度、扶養人数、課税対象金額から自動で税額を検索します。</x:v>
+        <x:v>CSV形式は `fiscalYear,dependentCount,minTaxable,maxTaxable,taxAmount` です。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="17" t="str">
-        <x:v>5. 給与入力</x:v>
-      </x:c>
-      <x:c r="B23" s="18" t="str"/>
-      <x:c r="C23" s="15" t="str"/>
+        <x:v>4. 所得税表</x:v>
+      </x:c>
+      <x:c r="B23" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>給与計算時は年度、扶養人数、課税対象金額から自動で税額を検索します。</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="17" t="str">
         <x:v>5. 給与入力</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C24" s="15" t="str">
-        <x:v>支給月を選択します。</x:v>
-      </x:c>
+      <x:c r="B24" s="18" t="str"/>
+      <x:c r="C24" s="15" t="str"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
         <x:v>5. 給与入力</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C25" s="15" t="str">
-        <x:v>社員を選択し、基本給、固定残業手当、手当、住民税、寮使用料、備考などを入力します。</x:v>
+        <x:v>「給与管理」から「給与入力」を開き、支給月を選択します。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -693,10 +693,10 @@
         <x:v>5. 給与入力</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C26" s="15" t="str">
-        <x:v>「前回利用」は選択中社員本人の過去入力だけを参照します。</x:v>
+        <x:v>社員を選択し、基本給、固定残業手当、手当、住民税、寮使用料、備考などを入力します。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -704,10 +704,10 @@
         <x:v>5. 給与入力</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="15" t="str">
-        <x:v>28日以降は前月以前の通常更新が制限されます。必要な場合は強制変更を選択して保存します。</x:v>
+        <x:v>「前回利用」は選択中社員本人の過去入力だけを参照します。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -715,39 +715,39 @@
         <x:v>5. 給与入力</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C28" s="15" t="str">
-        <x:v>支給日は会社運用に合わせ、システム日が25日以下の場合は前月を初期表示します。</x:v>
+        <x:v>28日以降は前月以前の通常更新が制限されます。必要な場合は強制変更を選択して保存します。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>6. 賞与入力</x:v>
-      </x:c>
-      <x:c r="B29" s="18" t="str"/>
-      <x:c r="C29" s="15" t="str"/>
+        <x:v>5. 給与入力</x:v>
+      </x:c>
+      <x:c r="B29" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>支給日は会社運用に合わせ、システム日が25日以下の場合は前月を初期表示します。</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
         <x:v>6. 賞与入力</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="15" t="str">
-        <x:v>月給とは別に賞与を登録します。</x:v>
-      </x:c>
+      <x:c r="B30" s="18" t="str"/>
+      <x:c r="C30" s="15" t="str"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
         <x:v>6. 賞与入力</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C31" s="15" t="str">
-        <x:v>賞与がない社員は登録不要です。</x:v>
+        <x:v>「給与管理」から「賞与入力」を開き、月給とは別に賞与を登録します。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
@@ -755,10 +755,10 @@
         <x:v>6. 賞与入力</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C32" s="15" t="str">
-        <x:v>通常賞与月は4月末、10月末を想定しています。</x:v>
+        <x:v>賞与がない社員は登録不要です。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -766,39 +766,39 @@
         <x:v>6. 賞与入力</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C33" s="15" t="str">
-        <x:v>賞与所得税は現状、給与と同じ所得税表ロジックで計算します。</x:v>
+        <x:v>通常賞与月は4月末、10月末を想定しています。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="17" t="str">
-        <x:v>7. PDF出力</x:v>
-      </x:c>
-      <x:c r="B34" s="18" t="str"/>
-      <x:c r="C34" s="15" t="str"/>
+        <x:v>6. 賞与入力</x:v>
+      </x:c>
+      <x:c r="B34" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>賞与所得税は現状、給与と同じ所得税表ロジックで計算します。</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>7. PDF出力</x:v>
       </x:c>
-      <x:c r="B35" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
-        <x:v>社員ごとの給与明細PDFをダウンロードできます。</x:v>
-      </x:c>
+      <x:c r="B35" s="18" t="str"/>
+      <x:c r="C35" s="15" t="str"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
         <x:v>7. PDF出力</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C36" s="15" t="str">
-        <x:v>指定月範囲で一括出力できます。</x:v>
+        <x:v>「給与管理」から「明細出力」を開き、社員ごとの給与明細PDFをダウンロードできます。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -806,10 +806,10 @@
         <x:v>7. PDF出力</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C37" s="15" t="str">
-        <x:v>出力方法は個別PDFまたは1つのPDFにまとめる方式を選択できます。</x:v>
+        <x:v>指定月範囲で一括出力できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -817,10 +817,10 @@
         <x:v>7. PDF出力</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C38" s="15" t="str">
-        <x:v>「賞与含み」にチェックした場合、対象期間の賞与明細も含めます。</x:v>
+        <x:v>出力方法は個別PDFまたは1つのPDFにまとめる方式を選択できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -828,144 +828,206 @@
         <x:v>7. PDF出力</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C39" s="15" t="str">
-        <x:v>ファイル名は給与明細が `給与明細_年月_名前`、一括出力が `給与明細_開始年月_終了年月` です。</x:v>
+        <x:v>「賞与含み」にチェックした場合、対象期間の賞与明細も含めます。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
-      </x:c>
-      <x:c r="B40" s="18" t="str"/>
-      <x:c r="C40" s="15" t="str"/>
+        <x:v>7. PDF出力</x:v>
+      </x:c>
+      <x:c r="B40" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C40" s="15" t="str">
+        <x:v>ファイル名は給与明細が `給与明細_年月_名前`、一括出力が `給与明細_開始年月_終了年月` です。</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
-      </x:c>
-      <x:c r="B41" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C41" s="15" t="str">
-        <x:v>「管理メニュー」からユーザ管理と権限管理を開きます。</x:v>
-      </x:c>
+        <x:v>7.1 給与管理メニュー</x:v>
+      </x:c>
+      <x:c r="B41" s="18" t="str"/>
+      <x:c r="C41" s="15" t="str"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
+        <x:v>7.1 給与管理メニュー</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C42" s="15" t="str">
-        <x:v>権限管理ではロール一覧、ロール追加、非表示、ロールごとのメニュー権限を設定できます。</x:v>
+        <x:v>給与管理は、給与・賞与入力、明細出力、社員管理、年度設定の子メニューで管理します。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
+        <x:v>7.1 給与管理メニュー</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C43" s="15" t="str">
-        <x:v>メニュー表示、閲覧、更新、全件、自分のみを子メニュー単位で設定できます。</x:v>
+        <x:v>権限がない子メニューは表示されません。</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
+        <x:v>7.1 給与管理メニュー</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C44" s="15" t="str">
-        <x:v>ユーザ登録時は利用可能なロールを選択し、必要に応じてユーザ個別の権限を上書きできます。</x:v>
+        <x:v>子メニューを切り替えると、前画面のメッセージはクリアされます。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="17" t="str">
-        <x:v>8. 権限管理</x:v>
+        <x:v>7.1 給与管理メニュー</x:v>
       </x:c>
       <x:c r="B45" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C45" s="15" t="str">
-        <x:v>権限管理では、給与管理、SES管理、管理メニューごとに表示、閲覧、更新、全件を一括チェックできます。</x:v>
+        <x:v>給与・賞与入力画面では、選択月の給与・賞与が登録済みか未登録かを社員一覧に表示します。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>8. 権限管理</x:v>
       </x:c>
-      <x:c r="B46" s="18" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C46" s="15" t="str">
-        <x:v>ロール保存や権限保存に失敗した場合、権限管理画面内にエラーメッセージが表示されます。</x:v>
-      </x:c>
+      <x:c r="B46" s="18" t="str"/>
+      <x:c r="C46" s="15" t="str"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="17" t="str">
-        <x:v>9. メッセージ表示</x:v>
-      </x:c>
-      <x:c r="B47" s="18" t="str"/>
-      <x:c r="C47" s="15" t="str"/>
+        <x:v>8. 権限管理</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C47" s="15" t="str">
+        <x:v>「管理メニュー」からユーザ管理と権限管理を開きます。</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="17" t="str">
-        <x:v>9. メッセージ表示</x:v>
+        <x:v>8. 権限管理</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="15" t="str">
-        <x:v>入力エラーや保存失敗などのエラーメッセージは、赤字で対象操作画面のメニュー直下に表示されます。</x:v>
+        <x:v>権限管理ではロール一覧、ロール追加、非表示、ロールごとのメニュー権限を設定できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="17" t="str">
-        <x:v>9. メッセージ表示</x:v>
+        <x:v>8. 権限管理</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C49" s="15" t="str">
-        <x:v>給与管理のエラーは給与管理メニュー直下、権限管理のエラーは権限管理画面内に表示されます。</x:v>
+        <x:v>メニュー表示、閲覧、更新、全件、自分のみを子メニュー単位で設定できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="17" t="str">
-        <x:v>9. メッセージ表示</x:v>
+        <x:v>8. 権限管理</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C50" s="15" t="str">
-        <x:v>保存、検索、PDF出力などの操作完了メッセージは、緑色のtoastで画面右上に表示され、自動で消えます。</x:v>
+        <x:v>ユーザ登録時は利用可能なロールを選択し、必要に応じてユーザ個別の権限を上書きできます。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="17" t="str">
-        <x:v>9. メッセージ表示</x:v>
+        <x:v>8. 権限管理</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C51" s="15" t="str">
-        <x:v>メニューを切り替えると、前の画面のメッセージはクリアされます。</x:v>
+        <x:v>権限管理では、給与管理、SES管理、管理メニューごとに表示、閲覧、更新、全件を一括チェックできます。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="17" t="str">
+        <x:v>8. 権限管理</x:v>
+      </x:c>
+      <x:c r="B52" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C52" s="15" t="str">
+        <x:v>ロール保存や権限保存に失敗した場合、権限管理画面内にエラーメッセージが表示されます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="17" t="str">
         <x:v>9. メッセージ表示</x:v>
       </x:c>
-      <x:c r="B52" s="18" t="n">
+      <x:c r="B53" s="18" t="str"/>
+      <x:c r="C53" s="15" t="str"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="17" t="str">
+        <x:v>9. メッセージ表示</x:v>
+      </x:c>
+      <x:c r="B54" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C54" s="15" t="str">
+        <x:v>入力エラーや保存失敗などのエラーメッセージは、赤字で対象操作画面のメニュー直下に表示されます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="17" t="str">
+        <x:v>9. メッセージ表示</x:v>
+      </x:c>
+      <x:c r="B55" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C55" s="15" t="str">
+        <x:v>給与管理のエラーは給与管理メニュー直下、権限管理のエラーは権限管理画面内に表示されます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="17" t="str">
+        <x:v>9. メッセージ表示</x:v>
+      </x:c>
+      <x:c r="B56" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C56" s="15" t="str">
+        <x:v>保存、検索、PDF出力などの操作完了メッセージは、緑色のtoastで画面右上に表示され、自動で消えます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="17" t="str">
+        <x:v>9. メッセージ表示</x:v>
+      </x:c>
+      <x:c r="B57" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C57" s="15" t="str">
+        <x:v>メニューを切り替えると、前の画面のメッセージはクリアされます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="17" t="str">
+        <x:v>9. メッセージ表示</x:v>
+      </x:c>
+      <x:c r="B58" s="18" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C52" s="15" t="str">
+      <x:c r="C58" s="15" t="str">
         <x:v>ログイン画面にはログイン失敗などログイン専用メッセージだけ表示されます。</x:v>
       </x:c>
     </x:row>
@@ -1071,7 +1133,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>从“工资管理”进入员工列表。</x:v>
+        <x:v>从“工资管理”进入“员工管理”。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1109,31 +1171,31 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="17" t="str">
-        <x:v>3. 年度和费率管理</x:v>
-      </x:c>
-      <x:c r="B14" s="18" t="str"/>
-      <x:c r="C14" s="15" t="str"/>
+        <x:v>2. 员工管理</x:v>
+      </x:c>
+      <x:c r="B14" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="str">
+        <x:v>可以按员工设置是否有奖金。有奖金时，最多可登记3次奖金的支付月份和金额。</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>3. 年度和费率管理</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C15" s="15" t="str">
-        <x:v>税率、社会保险费率按年度维护。</x:v>
-      </x:c>
+      <x:c r="B15" s="18" t="str"/>
+      <x:c r="C15" s="15" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
         <x:v>3. 年度和费率管理</x:v>
       </x:c>
       <x:c r="B16" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C16" s="15" t="str">
-        <x:v>健康护理保险、厚生年金、雇用保险、儿童育儿支援金分开录入。</x:v>
+        <x:v>税率、社会保险费率按年度维护。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1141,10 +1203,10 @@
         <x:v>3. 年度和费率管理</x:v>
       </x:c>
       <x:c r="B17" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C17" s="15" t="str">
-        <x:v>小数点最多支持6位。</x:v>
+        <x:v>健康护理保险、厚生年金、雇用保险、儿童育儿支援金分开录入。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1152,39 +1214,39 @@
         <x:v>3. 年度和费率管理</x:v>
       </x:c>
       <x:c r="B18" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C18" s="15" t="str">
-        <x:v>住民税在工资录入时按员工、月份录入。</x:v>
+        <x:v>小数点最多支持6位。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>4. 所得税表</x:v>
-      </x:c>
-      <x:c r="B19" s="18" t="str"/>
-      <x:c r="C19" s="15" t="str"/>
+        <x:v>3. 年度和费率管理</x:v>
+      </x:c>
+      <x:c r="B19" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>住民税在工资录入时按员工、月份录入。</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C20" s="15" t="str">
-        <x:v>导入所得税表CSV。</x:v>
-      </x:c>
+      <x:c r="B20" s="18" t="str"/>
+      <x:c r="C20" s="15" t="str"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
-        <x:v>CSV格式为 `fiscalYear,dependentCount,minTaxable,maxTaxable,taxAmount`。</x:v>
+        <x:v>导入所得税表CSV。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -1192,39 +1254,39 @@
         <x:v>4. 所得税表</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="15" t="str">
-        <x:v>计算工资时，系统按年度、扶养人数、课税对象金额自动查表。</x:v>
+        <x:v>CSV格式为 `fiscalYear,dependentCount,minTaxable,maxTaxable,taxAmount`。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="17" t="str">
-        <x:v>5. 工资录入</x:v>
-      </x:c>
-      <x:c r="B23" s="18" t="str"/>
-      <x:c r="C23" s="15" t="str"/>
+        <x:v>4. 所得税表</x:v>
+      </x:c>
+      <x:c r="B23" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>计算工资时，系统按年度、扶养人数、课税对象金额自动查表。</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="17" t="str">
         <x:v>5. 工资录入</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C24" s="15" t="str">
-        <x:v>选择支付月份。</x:v>
-      </x:c>
+      <x:c r="B24" s="18" t="str"/>
+      <x:c r="C24" s="15" t="str"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
         <x:v>5. 工资录入</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C25" s="15" t="str">
-        <x:v>选择员工，输入基本工资、固定加班补贴、补贴、住民税、宿舍费、备注等。</x:v>
+        <x:v>从“工资管理”进入“工资输入”，选择支付月份。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -1232,10 +1294,10 @@
         <x:v>5. 工资录入</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C26" s="15" t="str">
-        <x:v>“使用上次内容”只引用当前员工自己的历史录入。</x:v>
+        <x:v>选择员工，输入基本工资、固定加班补贴、补贴、住民税、宿舍费、备注等。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -1243,10 +1305,10 @@
         <x:v>5. 工资录入</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="15" t="str">
-        <x:v>28日以后，前月及以前数据默认不能普通更新。如需修改，选择强制变更后保存。</x:v>
+        <x:v>“使用上次内容”只引用当前员工自己的历史录入。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -1254,39 +1316,39 @@
         <x:v>5. 工资录入</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C28" s="15" t="str">
-        <x:v>按公司25日发上月工资的规则，系统日小于等于25日时默认显示前月。</x:v>
+        <x:v>28日以后，前月及以前数据默认不能普通更新。如需修改，选择强制变更后保存。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>6. 奖金录入</x:v>
-      </x:c>
-      <x:c r="B29" s="18" t="str"/>
-      <x:c r="C29" s="15" t="str"/>
+        <x:v>5. 工资录入</x:v>
+      </x:c>
+      <x:c r="B29" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>按公司25日发上月工资的规则，系统日小于等于25日时默认显示前月。</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
         <x:v>6. 奖金录入</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="15" t="str">
-        <x:v>奖金与月工资分开录入。</x:v>
-      </x:c>
+      <x:c r="B30" s="18" t="str"/>
+      <x:c r="C30" s="15" t="str"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
         <x:v>6. 奖金录入</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C31" s="15" t="str">
-        <x:v>没有奖金的员工无需录入。</x:v>
+        <x:v>从“工资管理”进入“奖金输入”，奖金与月工资分开录入。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
@@ -1294,10 +1356,10 @@
         <x:v>6. 奖金录入</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C32" s="15" t="str">
-        <x:v>通常奖金月份按4月底和10月底处理。</x:v>
+        <x:v>没有奖金的员工无需录入。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -1305,39 +1367,39 @@
         <x:v>6. 奖金录入</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C33" s="15" t="str">
-        <x:v>当前奖金所得税使用与工资相同的所得税表逻辑计算。</x:v>
+        <x:v>通常奖金月份按4月底和10月底处理。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="17" t="str">
-        <x:v>7. PDF输出</x:v>
-      </x:c>
-      <x:c r="B34" s="18" t="str"/>
-      <x:c r="C34" s="15" t="str"/>
+        <x:v>6. 奖金录入</x:v>
+      </x:c>
+      <x:c r="B34" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>当前奖金所得税使用与工资相同的所得税表逻辑计算。</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>7. PDF输出</x:v>
       </x:c>
-      <x:c r="B35" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
-        <x:v>可下载单个员工的工资明细PDF。</x:v>
-      </x:c>
+      <x:c r="B35" s="18" t="str"/>
+      <x:c r="C35" s="15" t="str"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
         <x:v>7. PDF输出</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C36" s="15" t="str">
-        <x:v>可按月份范围批量下载。</x:v>
+        <x:v>从“工资管理”进入“明细输出”，可下载单个员工的工资明细PDF。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -1345,10 +1407,10 @@
         <x:v>7. PDF输出</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C37" s="15" t="str">
-        <x:v>输出方式可选择多个PDF或合并成一个PDF。</x:v>
+        <x:v>可按月份范围批量下载。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -1356,10 +1418,10 @@
         <x:v>7. PDF输出</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C38" s="15" t="str">
-        <x:v>勾选“包含奖金”时，期间内的奖金明细也会一起输出。</x:v>
+        <x:v>输出方式可选择多个PDF或合并成一个PDF。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -1367,144 +1429,206 @@
         <x:v>7. PDF输出</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C39" s="15" t="str">
-        <x:v>文件名规则: 工资明细为 `給与明細_年月_姓名`，批量输出为 `給与明細_开始年月_结束年月`。</x:v>
+        <x:v>勾选“包含奖金”时，期间内的奖金明细也会一起输出。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
-      </x:c>
-      <x:c r="B40" s="18" t="str"/>
-      <x:c r="C40" s="15" t="str"/>
+        <x:v>7. PDF输出</x:v>
+      </x:c>
+      <x:c r="B40" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C40" s="15" t="str">
+        <x:v>文件名规则: 工资明细为 `給与明細_年月_姓名`，批量输出为 `給与明細_开始年月_结束年月`。</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
-      </x:c>
-      <x:c r="B41" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C41" s="15" t="str">
-        <x:v>从“管理菜单”进入用户管理和权限管理。</x:v>
-      </x:c>
+        <x:v>7.1 工资管理菜单</x:v>
+      </x:c>
+      <x:c r="B41" s="18" t="str"/>
+      <x:c r="C41" s="15" t="str"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
+        <x:v>7.1 工资管理菜单</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C42" s="15" t="str">
-        <x:v>权限管理支持角色列表、角色新增、隐藏、按角色设置菜单权限。</x:v>
+        <x:v>工资管理通过工资・奖金输入、明细输出、员工管理、年度设置等子菜单管理。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
+        <x:v>7.1 工资管理菜单</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C43" s="15" t="str">
-        <x:v>可以按子菜单设置是否显示、查看、更新、全件、自身数据。</x:v>
+        <x:v>没有权限的子菜单不会显示。</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
+        <x:v>7.1 工资管理菜单</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C44" s="15" t="str">
-        <x:v>用户注册时选择可用角色，必要时可以按用户单独覆盖菜单权限。</x:v>
+        <x:v>切换子菜单时，会清除前一个画面的消息。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="17" t="str">
-        <x:v>8. 权限管理</x:v>
+        <x:v>7.1 工资管理菜单</x:v>
       </x:c>
       <x:c r="B45" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C45" s="15" t="str">
-        <x:v>在权限管理中，可以按工资管理、SES管理、管理菜单为单位，一次勾选显示、查看、更新、全件。</x:v>
+        <x:v>在工资・奖金输入画面，员工列表会显示当前月份工资和奖金是否已登记。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>8. 权限管理</x:v>
       </x:c>
-      <x:c r="B46" s="18" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C46" s="15" t="str">
-        <x:v>角色保存或权限保存失败时，错误信息会显示在权限管理画面内。</x:v>
-      </x:c>
+      <x:c r="B46" s="18" t="str"/>
+      <x:c r="C46" s="15" t="str"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="17" t="str">
-        <x:v>9. 消息显示</x:v>
-      </x:c>
-      <x:c r="B47" s="18" t="str"/>
-      <x:c r="C47" s="15" t="str"/>
+        <x:v>8. 权限管理</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C47" s="15" t="str">
+        <x:v>从“管理菜单”进入用户管理和权限管理。</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="17" t="str">
-        <x:v>9. 消息显示</x:v>
+        <x:v>8. 权限管理</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="15" t="str">
-        <x:v>输入错误、保存失败等错误信息，以红字显示在对应操作画面的菜单下方。</x:v>
+        <x:v>权限管理支持角色列表、角色新增、隐藏、按角色设置菜单权限。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="17" t="str">
-        <x:v>9. 消息显示</x:v>
+        <x:v>8. 权限管理</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C49" s="15" t="str">
-        <x:v>工资管理的错误显示在工资管理菜单下方，权限管理的错误显示在权限管理画面内。</x:v>
+        <x:v>可以按子菜单设置是否显示、查看、更新、全件、自身数据。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="17" t="str">
-        <x:v>9. 消息显示</x:v>
+        <x:v>8. 权限管理</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C50" s="15" t="str">
-        <x:v>保存、搜索、PDF输出等操作完成消息，以绿色 toast 显示在画面右上，并自动消失。</x:v>
+        <x:v>用户注册时选择可用角色，必要时可以按用户单独覆盖菜单权限。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="17" t="str">
-        <x:v>9. 消息显示</x:v>
+        <x:v>8. 权限管理</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C51" s="15" t="str">
-        <x:v>切换菜单时，会清除前一个画面的消息。</x:v>
+        <x:v>在权限管理中，可以按工资管理、SES管理、管理菜单为单位，一次勾选显示、查看、更新、全件。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="17" t="str">
+        <x:v>8. 权限管理</x:v>
+      </x:c>
+      <x:c r="B52" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C52" s="15" t="str">
+        <x:v>角色保存或权限保存失败时，错误信息会显示在权限管理画面内。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="17" t="str">
         <x:v>9. 消息显示</x:v>
       </x:c>
-      <x:c r="B52" s="18" t="n">
+      <x:c r="B53" s="18" t="str"/>
+      <x:c r="C53" s="15" t="str"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="17" t="str">
+        <x:v>9. 消息显示</x:v>
+      </x:c>
+      <x:c r="B54" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C54" s="15" t="str">
+        <x:v>输入错误、保存失败等错误信息，以红字显示在对应操作画面的菜单下方。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="17" t="str">
+        <x:v>9. 消息显示</x:v>
+      </x:c>
+      <x:c r="B55" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C55" s="15" t="str">
+        <x:v>工资管理的错误显示在工资管理菜单下方，权限管理的错误显示在权限管理画面内。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="17" t="str">
+        <x:v>9. 消息显示</x:v>
+      </x:c>
+      <x:c r="B56" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C56" s="15" t="str">
+        <x:v>保存、搜索、PDF输出等操作完成消息，以绿色 toast 显示在画面右上，并自动消失。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="17" t="str">
+        <x:v>9. 消息显示</x:v>
+      </x:c>
+      <x:c r="B57" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C57" s="15" t="str">
+        <x:v>切换菜单时，会清除前一个画面的消息。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="17" t="str">
+        <x:v>9. 消息显示</x:v>
+      </x:c>
+      <x:c r="B58" s="18" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C52" s="15" t="str">
+      <x:c r="C58" s="15" t="str">
         <x:v>登录画面只显示登录失败等登录专用消息。</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Restore employee slips on payroll output
</commit_message>
<xml_diff>
--- a/docs/manual_payroll_ses_ja_zh.xlsx
+++ b/docs/manual_payroll_ses_ja_zh.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目次" sheetId="1" r:id="R53edcda026ec49bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_JA" sheetId="2" r:id="R31b16f3e071a4a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_ZH" sheetId="3" r:id="R596937e65c6f4d07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_JA" sheetId="4" r:id="R1798e802ae414602"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_ZH" sheetId="5" r:id="R0c6ed986ab2e4167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目次" sheetId="1" r:id="R7c15d3ae57f04cf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_JA" sheetId="2" r:id="Rac90c7ee92394866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="給与_ZH" sheetId="3" r:id="Rfc6cf74c0ed9456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_JA" sheetId="4" r:id="Rc8e75fff60684fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SES_ZH" sheetId="5" r:id="R7fc8e6dab8274625"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -465,7 +465,11 @@
         <x:v>更新日: 2026-07-26</x:v>
       </x:c>
     </x:row>
-    <x:row r="3"/>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+    </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>セクション</x:v>
@@ -481,8 +485,8 @@
       <x:c r="A5" s="17" t="str">
         <x:v>1. ログイン</x:v>
       </x:c>
-      <x:c r="B5" s="18" t="str"/>
-      <x:c r="C5" s="15" t="str"/>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="15"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -521,8 +525,8 @@
       <x:c r="A9" s="17" t="str">
         <x:v>2. 社員管理</x:v>
       </x:c>
-      <x:c r="B9" s="18" t="str"/>
-      <x:c r="C9" s="15" t="str"/>
+      <x:c r="B9" s="18"/>
+      <x:c r="C9" s="15"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -583,8 +587,8 @@
       <x:c r="A15" s="17" t="str">
         <x:v>3. 年度・料率管理</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="str"/>
-      <x:c r="C15" s="15" t="str"/>
+      <x:c r="B15" s="18"/>
+      <x:c r="C15" s="15"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -634,8 +638,8 @@
       <x:c r="A20" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str"/>
-      <x:c r="C20" s="15" t="str"/>
+      <x:c r="B20" s="18"/>
+      <x:c r="C20" s="15"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
@@ -674,8 +678,8 @@
       <x:c r="A24" s="17" t="str">
         <x:v>5. 給与入力</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="str"/>
-      <x:c r="C24" s="15" t="str"/>
+      <x:c r="B24" s="18"/>
+      <x:c r="C24" s="15"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
@@ -736,8 +740,8 @@
       <x:c r="A30" s="17" t="str">
         <x:v>6. 賞与入力</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="str"/>
-      <x:c r="C30" s="15" t="str"/>
+      <x:c r="B30" s="18"/>
+      <x:c r="C30" s="15"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
@@ -787,8 +791,8 @@
       <x:c r="A35" s="17" t="str">
         <x:v>7. PDF出力</x:v>
       </x:c>
-      <x:c r="B35" s="18" t="str"/>
-      <x:c r="C35" s="15" t="str"/>
+      <x:c r="B35" s="18"/>
+      <x:c r="C35" s="15"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -798,7 +802,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C36" s="15" t="str">
-        <x:v>「給与管理」から「明細出力」を開き、社員ごとの給与明細PDFをダウンロードできます。</x:v>
+        <x:v>「給与管理」から「明細出力」を開くと、社員一覧で社員を選択し、給与明細・賞与明細を確認できます。期間指定のPDF一括ダウンロード、給与CSV、賞与CSVも同じ画面で出力できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -849,8 +853,8 @@
       <x:c r="A41" s="17" t="str">
         <x:v>7.1 給与管理メニュー</x:v>
       </x:c>
-      <x:c r="B41" s="18" t="str"/>
-      <x:c r="C41" s="15" t="str"/>
+      <x:c r="B41" s="18"/>
+      <x:c r="C41" s="15"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -893,15 +897,15 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C45" s="15" t="str">
-        <x:v>給与・賞与入力画面では、選択月の給与・賞与が登録済みか未登録かを社員一覧に表示します。</x:v>
+        <x:v>給与・賞与入力画面と明細出力画面では、選択月の給与・賞与が登録済みか未登録かを社員一覧に表示します。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>8. 権限管理</x:v>
       </x:c>
-      <x:c r="B46" s="18" t="str"/>
-      <x:c r="C46" s="15" t="str"/>
+      <x:c r="B46" s="18"/>
+      <x:c r="C46" s="15"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="17" t="str">
@@ -973,8 +977,8 @@
       <x:c r="A53" s="17" t="str">
         <x:v>9. メッセージ表示</x:v>
       </x:c>
-      <x:c r="B53" s="18" t="str"/>
-      <x:c r="C53" s="15" t="str"/>
+      <x:c r="B53" s="18"/>
+      <x:c r="C53" s="15"/>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="17" t="str">
@@ -1066,7 +1070,11 @@
         <x:v>更新日: 2026-07-26</x:v>
       </x:c>
     </x:row>
-    <x:row r="3"/>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+    </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>セクション</x:v>
@@ -1082,8 +1090,8 @@
       <x:c r="A5" s="17" t="str">
         <x:v>1. 登录</x:v>
       </x:c>
-      <x:c r="B5" s="18" t="str"/>
-      <x:c r="C5" s="15" t="str"/>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="15"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -1122,8 +1130,8 @@
       <x:c r="A9" s="17" t="str">
         <x:v>2. 员工管理</x:v>
       </x:c>
-      <x:c r="B9" s="18" t="str"/>
-      <x:c r="C9" s="15" t="str"/>
+      <x:c r="B9" s="18"/>
+      <x:c r="C9" s="15"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -1184,8 +1192,8 @@
       <x:c r="A15" s="17" t="str">
         <x:v>3. 年度和费率管理</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="str"/>
-      <x:c r="C15" s="15" t="str"/>
+      <x:c r="B15" s="18"/>
+      <x:c r="C15" s="15"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -1235,8 +1243,8 @@
       <x:c r="A20" s="17" t="str">
         <x:v>4. 所得税表</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str"/>
-      <x:c r="C20" s="15" t="str"/>
+      <x:c r="B20" s="18"/>
+      <x:c r="C20" s="15"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
@@ -1275,8 +1283,8 @@
       <x:c r="A24" s="17" t="str">
         <x:v>5. 工资录入</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="str"/>
-      <x:c r="C24" s="15" t="str"/>
+      <x:c r="B24" s="18"/>
+      <x:c r="C24" s="15"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
@@ -1337,8 +1345,8 @@
       <x:c r="A30" s="17" t="str">
         <x:v>6. 奖金录入</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="str"/>
-      <x:c r="C30" s="15" t="str"/>
+      <x:c r="B30" s="18"/>
+      <x:c r="C30" s="15"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
@@ -1388,8 +1396,8 @@
       <x:c r="A35" s="17" t="str">
         <x:v>7. PDF输出</x:v>
       </x:c>
-      <x:c r="B35" s="18" t="str"/>
-      <x:c r="C35" s="15" t="str"/>
+      <x:c r="B35" s="18"/>
+      <x:c r="C35" s="15"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -1399,7 +1407,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C36" s="15" t="str">
-        <x:v>从“工资管理”进入“明细输出”，可下载单个员工的工资明细PDF。</x:v>
+        <x:v>从“工资管理”进入“明细输出”后，可以在员工列表中选择员工，查看工资明细和奖金明细。期间指定的PDF批量下载、工资CSV、奖金CSV也在同一画面输出。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -1450,8 +1458,8 @@
       <x:c r="A41" s="17" t="str">
         <x:v>7.1 工资管理菜单</x:v>
       </x:c>
-      <x:c r="B41" s="18" t="str"/>
-      <x:c r="C41" s="15" t="str"/>
+      <x:c r="B41" s="18"/>
+      <x:c r="C41" s="15"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -1494,15 +1502,15 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C45" s="15" t="str">
-        <x:v>在工资・奖金输入画面，员工列表会显示当前月份工资和奖金是否已登记。</x:v>
+        <x:v>在工资・奖金输入画面和明细输出画面，员工列表会显示当前月份工资和奖金是否已登记。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>8. 权限管理</x:v>
       </x:c>
-      <x:c r="B46" s="18" t="str"/>
-      <x:c r="C46" s="15" t="str"/>
+      <x:c r="B46" s="18"/>
+      <x:c r="C46" s="15"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="17" t="str">
@@ -1574,8 +1582,8 @@
       <x:c r="A53" s="17" t="str">
         <x:v>9. 消息显示</x:v>
       </x:c>
-      <x:c r="B53" s="18" t="str"/>
-      <x:c r="C53" s="15" t="str"/>
+      <x:c r="B53" s="18"/>
+      <x:c r="C53" s="15"/>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="17" t="str">

</xml_diff>